<commit_message>
Domain_Coverage: separate 'not a Findings domain'
Events, Interventions, Special-Purpose and Trial Design domains get their
own status instead of 'no consumer class assigned' / 'no content': the
three files are Findings consumers, so no rule could place them. 'no
consumer class assigned' now lists only Findings domains (21);
'no content' only PE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzSyuaqVq1B4PFnRpWB
</commit_message>
<xml_diff>
--- a/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
+++ b/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-29 20:42</t>
+          <t>Generated: 2026-10-29 20:45</t>
         </is>
       </c>
     </row>
@@ -675,107 +675,121 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>no content — no test codes and no DSSs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+          <t>not a Findings domain — Observation_Class is not Findings; the three files are Findings consumers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>no content — a Findings domain with no test codes and no DSSs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>SUMMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  covered: 10 domains, 662 DSSs</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  in scope, no DSS: 6 domains, 0 DSSs</t>
+          <t xml:space="preserve">  covered: 10 domains, 662 DSSs</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  excluded: 2 domains, 364 DSSs</t>
+          <t xml:space="preserve">  in scope, no DSS: 6 domains, 0 DSSs</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  no consumer class assigned: 32 domains, 449 DSSs</t>
+          <t xml:space="preserve">  excluded: 2 domains, 364 DSSs</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  no content: 16 domains, 0 DSSs</t>
+          <t xml:space="preserve">  no consumer class assigned: 21 domains, 238 DSSs</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  not a Findings domain: 26 domains, 211 DSSs</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  no content: 1 domains, 0 DSSs</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  DSS total 1,475 = DSS_View Measurement_Specs.</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>CHECKS (the run fails otherwise)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Every domain in a Findings file is in that consumer's computed scope.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>Every covered domain has all its DSS_View DSSs in its Findings file.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
+          <t>Every domain in a Findings file is in that consumer's computed scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Every covered domain has all its DSS_View DSSs in its Findings file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
           <t>Every domain with content is in SDTM_Domain_Metadata; no domain is in two consumer classes.</t>
         </is>
       </c>
     </row>
-    <row r="47"/>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>HEADER COLOUR CONVENTION</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>Green = SDTM-CT side (TESTCD_Count). Yellow = COSMoS side (DSS_Count). Grey = keys, metadata, status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Green = SDTM-CT side (TESTCD_Count). Yellow = COSMoS side (DSS_Count). Grey = keys, metadata, status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Not an official CDISC product.</t>
         </is>
@@ -1682,29 +1696,29 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Adverse Events</t>
+          <t>Auricular Findings</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="7" t="n">
@@ -1716,17 +1730,21 @@
         </is>
       </c>
       <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>DA</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Auricular Findings</t>
+          <t>Drug Accountability</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1740,7 +1758,7 @@
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F21" s="7" t="n">
         <v>0</v>
@@ -1755,38 +1773,34 @@
         </is>
       </c>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
-        </is>
-      </c>
+      <c r="K21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DD</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Biospecimen Events</t>
+          <t>Death Details</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G22" s="7" t="n"/>
       <c r="H22" s="7" t="n">
@@ -1798,38 +1812,34 @@
         </is>
       </c>
       <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>From SDTMIG-PGx v1.0</t>
-        </is>
-      </c>
+      <c r="K22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>CM</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Concomitant/Prior Medications</t>
+          <t>Device Properties</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G23" s="7" t="n"/>
       <c r="H23" s="7" t="n">
@@ -1841,17 +1851,21 @@
         </is>
       </c>
       <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Device characteristics, not an observation of the subject: no consumer class.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>DA</t>
+          <t>DU</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Drug Accountability</t>
+          <t>Device In-Use</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1865,7 +1879,7 @@
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>6</v>
+        <v>67</v>
       </c>
       <c r="F24" s="7" t="n">
         <v>0</v>
@@ -1880,17 +1894,21 @@
         </is>
       </c>
       <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Device settings in use, not an observation of the subject: no consumer class.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>DD</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Death Details</t>
+          <t>Endocrine System Findings</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -1904,10 +1922,10 @@
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n">
@@ -1919,34 +1937,38 @@
         </is>
       </c>
       <c r="J25" s="7" t="n"/>
-      <c r="K25" s="7" t="n"/>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Findings About Events or Interventions</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Special-Purpose</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G26" s="7" t="n"/>
       <c r="H26" s="7" t="n">
@@ -1963,12 +1985,12 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>GI</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Device Properties</t>
+          <t>Gastrointestinal System Findings</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -1982,7 +2004,7 @@
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F27" s="7" t="n">
         <v>0</v>
@@ -1999,36 +2021,36 @@
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Device characteristics, not an observation of the subject: no consumer class.</t>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>HM</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Disposition</t>
+          <t>Hematopoietic System Findings</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G28" s="7" t="n"/>
       <c r="H28" s="7" t="n">
@@ -2040,17 +2062,21 @@
         </is>
       </c>
       <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>DU</t>
+          <t>IE</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Device In-Use</t>
+          <t>Inclusion/Exclusion Criteria Not Met</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -2064,10 +2090,10 @@
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n">
@@ -2079,38 +2105,34 @@
         </is>
       </c>
       <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="inlineStr">
-        <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Device settings in use, not an observation of the subject: no consumer class.</t>
-        </is>
-      </c>
+      <c r="K29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Exposure as Collected</t>
+          <t>Integumentary System Findings</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G30" s="7" t="n"/>
       <c r="H30" s="7" t="n">
@@ -2122,17 +2144,21 @@
         </is>
       </c>
       <c r="J30" s="7" t="n"/>
-      <c r="K30" s="7" t="n"/>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Endocrine System Findings</t>
+          <t>Nervous System Findings</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -2146,7 +2172,7 @@
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>2</v>
+        <v>89</v>
       </c>
       <c r="F31" s="7" t="n">
         <v>0</v>
@@ -2163,36 +2189,36 @@
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
+          <t>In SDTMIG v3.4 (6.3.7.4). Listed here first on 2026-10-01 from SDTM CT C66734 as a domain not in the IG; corrected 2026-10-12. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>OE</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Exposure</t>
+          <t>Ophthalmic Examinations</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="7" t="n"/>
       <c r="H32" s="7" t="n">
@@ -2204,17 +2230,21 @@
         </is>
       </c>
       <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>In SDTMIG v3.4 (6.3.7.5). Listed here first on 2026-10-01 from SDTM CT C66734 as a domain not in the IG; corrected 2026-10-12. Consumer class pending published COSMoS content.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Findings About Events or Interventions</t>
+          <t>Tobacco Product Testing</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -2228,10 +2258,10 @@
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G33" s="7" t="n"/>
       <c r="H33" s="7" t="n">
@@ -2243,17 +2273,21 @@
         </is>
       </c>
       <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Tobacco product sample testing, not an observation of the subject: no consumer class.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>GI</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Gastrointestinal System Findings</t>
+          <t>Reproductive System Findings</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -2267,10 +2301,10 @@
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>24</v>
+        <v>119</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="G34" s="7" t="n"/>
       <c r="H34" s="7" t="n">
@@ -2282,21 +2316,17 @@
         </is>
       </c>
       <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="inlineStr">
-        <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
-        </is>
-      </c>
+      <c r="K34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>HM</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Hematopoietic System Findings</t>
+          <t>Subject Characteristics</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -2310,10 +2340,10 @@
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="n">
@@ -2325,21 +2355,17 @@
         </is>
       </c>
       <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="inlineStr">
-        <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
-        </is>
-      </c>
+      <c r="K35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>SR</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Inclusion/Exclusion Criteria Not Met</t>
+          <t>Skin Response</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -2353,10 +2379,10 @@
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F36" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G36" s="7" t="n"/>
       <c r="H36" s="7" t="n">
@@ -2373,12 +2399,12 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Integumentary System Findings</t>
+          <t>Subject Status</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -2392,7 +2418,7 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37" s="7" t="n">
         <v>0</v>
@@ -2407,38 +2433,34 @@
         </is>
       </c>
       <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="inlineStr">
-        <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
-        </is>
-      </c>
+      <c r="K37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Medical History</t>
+          <t>Tumor/Lesion Results</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G38" s="7" t="n"/>
       <c r="H38" s="7" t="n">
@@ -2450,17 +2472,21 @@
         </is>
       </c>
       <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>Oncology</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>NV</t>
+          <t>TU</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Nervous System Findings</t>
+          <t>Tumor/Lesion Identification</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -2474,10 +2500,10 @@
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n">
@@ -2491,19 +2517,19 @@
       <c r="J39" s="7" t="n"/>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>In SDTMIG v3.4 (6.3.7.4). Listed here first on 2026-10-01 from SDTM CT C66734 as a domain not in the IG; corrected 2026-10-12. Consumer class pending published COSMoS content.</t>
+          <t>Oncology</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>OE</t>
+          <t>UR</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Ophthalmic Examinations</t>
+          <t>Urinary System Findings</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -2517,10 +2543,10 @@
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G40" s="7" t="n"/>
       <c r="H40" s="7" t="n">
@@ -2532,26 +2558,22 @@
         </is>
       </c>
       <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="inlineStr">
-        <is>
-          <t>In SDTMIG v3.4 (6.3.7.5). Listed here first on 2026-10-01 from SDTM CT C66734 as a domain not in the IG; corrected 2026-10-12. Consumer class pending published COSMoS content.</t>
-        </is>
-      </c>
+      <c r="K40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>AE</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Procedures</t>
+          <t>Adverse Events</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -2563,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G41" s="7" t="n"/>
       <c r="H41" s="7" t="n">
@@ -2571,7 +2593,7 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J41" s="7" t="n"/>
@@ -2580,26 +2602,26 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>AG</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Tobacco Product Testing</t>
+          <t>Procedure Agents</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="F42" s="7" t="n">
         <v>0</v>
@@ -2610,42 +2632,38 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J42" s="7" t="n"/>
-      <c r="K42" s="7" t="inlineStr">
-        <is>
-          <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Tobacco product sample testing, not an observation of the subject: no consumer class.</t>
-        </is>
-      </c>
+      <c r="K42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Reproductive System Findings</t>
+          <t>Biospecimen Events</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>94</v>
+        <v>7</v>
       </c>
       <c r="G43" s="7" t="n"/>
       <c r="H43" s="7" t="n">
@@ -2653,38 +2671,42 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>From SDTMIG-PGx v1.0</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Subject Characteristics</t>
+          <t>Clinical Events</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="G44" s="7" t="n"/>
       <c r="H44" s="7" t="n">
@@ -2692,7 +2714,7 @@
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J44" s="7" t="n"/>
@@ -2701,29 +2723,29 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>CM</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Skin Response</t>
+          <t>Concomitant/Prior Medications</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G45" s="7" t="n"/>
       <c r="H45" s="7" t="n">
@@ -2731,7 +2753,7 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J45" s="7" t="n"/>
@@ -2740,26 +2762,26 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Subject Status</t>
+          <t>Comments</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Special-Purpose</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F46" s="7" t="n">
         <v>0</v>
@@ -2770,7 +2792,7 @@
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J46" s="7" t="n"/>
@@ -2779,17 +2801,17 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>SU</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Substance Use</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Special-Purpose</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -2801,7 +2823,7 @@
         <v>0</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G47" s="7" t="n"/>
       <c r="H47" s="7" t="n">
@@ -2809,7 +2831,7 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J47" s="7" t="n"/>
@@ -2818,29 +2840,29 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Tumor/Lesion Results</t>
+          <t>Disposition</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n">
@@ -2848,30 +2870,26 @@
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="inlineStr">
-        <is>
-          <t>Oncology</t>
-        </is>
-      </c>
+      <c r="K48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>DV</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Trial Summary</t>
+          <t>Protocol Deviations</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Trial Design</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -2883,7 +2901,7 @@
         <v>0</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="G49" s="7" t="n"/>
       <c r="H49" s="7" t="n">
@@ -2891,7 +2909,7 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J49" s="7" t="n"/>
@@ -2900,29 +2918,29 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>TU</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Tumor/Lesion Identification</t>
+          <t>Exposure as Collected</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G50" s="7" t="n"/>
       <c r="H50" s="7" t="n">
@@ -2930,42 +2948,38 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J50" s="7" t="n"/>
-      <c r="K50" s="7" t="inlineStr">
-        <is>
-          <t>Oncology</t>
-        </is>
-      </c>
+      <c r="K50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>EX</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Urinary System Findings</t>
+          <t>Exposure</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G51" s="7" t="n"/>
       <c r="H51" s="7" t="n">
@@ -2973,7 +2987,7 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>no consumer class assigned</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J51" s="7" t="n"/>
@@ -2982,17 +2996,17 @@
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>AG</t>
+          <t>HO</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Procedure Agents</t>
+          <t>Healthcare Encounters</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -3012,7 +3026,7 @@
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J52" s="7" t="n"/>
@@ -3021,12 +3035,12 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Clinical Events</t>
+          <t>Medical History</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -3043,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G53" s="7" t="n"/>
       <c r="H53" s="7" t="n">
@@ -3051,7 +3065,7 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J53" s="7" t="n"/>
@@ -3060,17 +3074,17 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Meal Data</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Special-Purpose</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -3090,26 +3104,30 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>New in v3.4 scope</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>DV</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Protocol Deviations</t>
+          <t>Procedures</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -3121,7 +3139,7 @@
         <v>0</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G55" s="7" t="n"/>
       <c r="H55" s="7" t="n">
@@ -3129,7 +3147,7 @@
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J55" s="7" t="n"/>
@@ -3138,17 +3156,17 @@
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Healthcare Encounters</t>
+          <t>Subject Elements</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Special-Purpose</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -3168,7 +3186,7 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J56" s="7" t="n"/>
@@ -3177,17 +3195,17 @@
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>SM</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Meal Data</t>
+          <t>Subject Disease Milestones</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Interventions</t>
+          <t>Special-Purpose</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -3207,42 +3225,38 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J57" s="7" t="n"/>
-      <c r="K57" s="7" t="inlineStr">
-        <is>
-          <t>New in v3.4 scope</t>
-        </is>
-      </c>
+      <c r="K57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>SU</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Physical Examination</t>
+          <t>Substance Use</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Interventions</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F58" s="7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G58" s="7" t="n"/>
       <c r="H58" s="7" t="n">
@@ -3250,25 +3264,21 @@
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J58" s="7" t="n"/>
-      <c r="K58" s="7" t="inlineStr">
-        <is>
-          <t>Added 2026-10-12 from SDTMIG v3.4.</t>
-        </is>
-      </c>
+      <c r="K58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Subject Elements</t>
+          <t>Subject Visits</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -3293,7 +3303,7 @@
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J59" s="7" t="n"/>
@@ -3302,17 +3312,17 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>SM</t>
+          <t>TA</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Subject Disease Milestones</t>
+          <t>Trial Arms</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Special-Purpose</t>
+          <t>Trial Design</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -3332,7 +3342,7 @@
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J60" s="7" t="n"/>
@@ -3341,17 +3351,17 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Subject Visits</t>
+          <t>Trial Disease Assessments</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Special-Purpose</t>
+          <t>Trial Design</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -3371,7 +3381,7 @@
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J61" s="7" t="n"/>
@@ -3380,12 +3390,12 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>TA</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Trial Arms</t>
+          <t>Trial Elements</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
@@ -3410,7 +3420,7 @@
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J62" s="7" t="n"/>
@@ -3419,12 +3429,12 @@
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>TD</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Trial Disease Assessments</t>
+          <t>Trial Inclusion/Exclusion Criteria</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -3449,7 +3459,7 @@
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J63" s="7" t="n"/>
@@ -3458,12 +3468,12 @@
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>TM</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Trial Elements</t>
+          <t>Trial Disease Milestones</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
@@ -3488,21 +3498,25 @@
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J64" s="7" t="n"/>
-      <c r="K64" s="7" t="n"/>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Added 2026-10-12 from SDTMIG v3.4.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Trial Inclusion/Exclusion Criteria</t>
+          <t>Trial Summary</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -3519,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="G65" s="7" t="n"/>
       <c r="H65" s="7" t="n">
@@ -3527,7 +3541,7 @@
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J65" s="7" t="n"/>
@@ -3536,12 +3550,12 @@
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>TM</t>
+          <t>TV</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Trial Disease Milestones</t>
+          <t>Trial Visits</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -3566,35 +3580,31 @@
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>no content</t>
+          <t>not a Findings domain</t>
         </is>
       </c>
       <c r="J66" s="7" t="n"/>
-      <c r="K66" s="7" t="inlineStr">
-        <is>
-          <t>Added 2026-10-12 from SDTMIG v3.4.</t>
-        </is>
-      </c>
+      <c r="K66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>TV</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Trial Visits</t>
+          <t>Physical Examination</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Trial Design</t>
+          <t>Findings</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
@@ -3613,7 +3623,11 @@
         </is>
       </c>
       <c r="J67" s="7" t="n"/>
-      <c r="K67" s="7" t="n"/>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>Added 2026-10-12 from SDTMIG v3.4.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>

</xml_diff>

<commit_message>
Findings round 3: instrument reference flag, DSS_Codelists, evaluated counts
Instrument_Findings: NCIt_Reference_Disagree for pinned instrument items is
compared against SDTM_Instrument_Test_Identity on TESTCD + Codelist_TESTCD
(DSS_View has no reference row for them); 171 rows now evaluated, none
disagree. Domain_Coverage: DSS_Codelists names the codelists the DSSs of
domains outside a consumer use (terms in COSMoS_Graph_CT, checked);
Reason states the flag values for domains no consumer rule places.
KNOWN GAPS in the three Findings files: how many rows each flag is
evaluated on, and how many are flagged Yes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzSyuaqVq1B4PFnRpWB
</commit_message>
<xml_diff>
--- a/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
+++ b/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain_Coverage" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Domain_Coverage'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Domain_Coverage'!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A71"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-29 21:33</t>
+          <t>Generated: 2026-10-29 21:53</t>
         </is>
       </c>
     </row>
@@ -597,307 +597,335 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  cosmos-graph/interim/COSMoS_Graph_CT.xlsx (CodelistTerms — to check that DSS_Codelists have terms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  sdtm-findings-graph/machine_actionable/Specimen_Findings.xlsx, Measurement_Findings.xlsx, Instrument_Findings.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>KNOWN GAPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>TESTCD_Count counts a test code once in every domain it belongs to; the column total is not a</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
+          <t>TESTCD_Count counts a test code once in every domain it belongs to; the column total is not a</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  count of distinct test codes.</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>SHEETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>ReadMe — this sheet.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>ReadMe — this sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>Domain_Coverage — one row per domain (see COLUMNS and COVERAGE STATUS).</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>COLUMNS</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Domain, Domain_Name, Observation_Class, Has_Test_Codes — SDTM_Domain_Metadata Domains.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Has_Test_Codes = the domain has a --TESTCD variable; CT need not have a codelist for it (IE, PC).</t>
+          <t>Domain, Domain_Name, Observation_Class, Has_Test_Codes — SDTM_Domain_Metadata Domains.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>TESTCD_Count — rows in SDTM_Test_Identity (domain in SDTM_Domains) plus SDTM_Instrument_Test_Identity.</t>
+          <t xml:space="preserve">  Has_Test_Codes = the domain has a --TESTCD variable; CT need not have a codelist for it (IE, PC).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>DSS_Count — COSMoS Dataset Specializations in DSS_View for the domain.</t>
+          <t>TESTCD_Count — rows in SDTM_Test_Identity (domain in SDTM_Domains) plus SDTM_Instrument_Test_Identity.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Consumer — the Findings file whose scope holds the domain, by the consumers' own rules</t>
+          <t>DSS_Count — COSMoS Dataset Specializations in DSS_View for the domain.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Specimen_Based, Measurement, Instrument_Domain_Rules, minus Consumer_Exclusions).</t>
+          <t>Consumer — the Findings file whose scope holds the domain, by the consumers' own rules</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>DSS_In_Consumer — DSS rows for the domain in that file's Measurement_Specs.</t>
+          <t xml:space="preserve">  (Specimen_Based, Measurement, Instrument_Domain_Rules, minus Consumer_Exclusions).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Coverage_Status — see below. Where_To_Look — the files and sheets that hold the domain's test codes and</t>
+          <t>DSS_In_Consumer — DSS rows for the domain in that file's Measurement_Specs.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSSs, from the counts: the consumer file; else SDTM_Test_Identity, SDTM_Instrument_Test_Identity,</t>
+          <t>Coverage_Status — see below. Where_To_Look — the files and sheets that hold the domain's test codes and</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSS_View (interim); or none in these files.</t>
+          <t xml:space="preserve">  DSSs, from the counts: the consumer file; else SDTM_Test_Identity, SDTM_Instrument_Test_Identity,</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Reason — the Consumer_Exclusions claim and reason for excluded domains; what is missing for in-scope</t>
+          <t xml:space="preserve">  DSS_View (interim); or none in these files.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  domains without DSSs.</t>
+          <t>DSS_Codelists — for domains with DSSs outside a consumer file: the codelists those DSSs name; their</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Domain_Notes — the Notes column of SDTM_Domain_Metadata Domains, as written there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45"/>
+          <t xml:space="preserve">  terms are in COSMoS_Graph_CT (interim), sheet CodelistTerms. Covered domains: see the Codelists sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of their Findings file.</t>
+        </is>
+      </c>
+    </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>COVERAGE STATUS</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Reason — the Consumer_Exclusions claim and reason for excluded domains; what is missing for in-scope</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>covered — in a consumer's scope; all its DSSs are in that file.</t>
+          <t xml:space="preserve">  domains without DSSs; the flag values for domains no consumer rule places.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>in scope, no DSS — in a consumer's scope; COSMoS has no DSS for it (Test_Identity only, if any).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>excluded — named in Consumer_Exclusions; the one status that rests on a recorded decision.</t>
-        </is>
-      </c>
-    </row>
+          <t>Domain_Notes — the Notes column of SDTM_Domain_Metadata Domains, as written there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>no consumer class assigned — has test codes or DSSs, but no consumer rule places it. A fact, not a decision.</t>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>COVERAGE STATUS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>not a Findings domain — Observation_Class is not Findings; the three files are Findings consumers.</t>
+          <t>covered — in a consumer's scope; all its DSSs are in that file.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>no content — a Findings domain with no test codes and no DSSs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53"/>
+          <t>in scope, no DSS — in a consumer's scope; COSMoS has no DSS for it (Test_Identity only, if any).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>excluded — named in Consumer_Exclusions; the one status that rests on a recorded decision.</t>
+        </is>
+      </c>
+    </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>SUMMARY</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>no consumer class assigned — has test codes or DSSs, but no consumer rule places it. A fact, not a decision.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  covered: 10 domains, 662 DSSs</t>
+          <t>not a Findings domain — Observation_Class is not Findings; the three files are Findings consumers.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  in scope, no DSS: 6 domains, 0 DSSs</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  excluded: 2 domains, 364 DSSs</t>
-        </is>
-      </c>
-    </row>
+          <t>no content — a Findings domain with no test codes and no DSSs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  no consumer class assigned: 21 domains, 238 DSSs</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  not a Findings domain: 26 domains, 211 DSSs</t>
+          <t xml:space="preserve">  covered: 10 domains, 662 DSSs</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  no content: 1 domains, 0 DSSs</t>
+          <t xml:space="preserve">  in scope, no DSS: 6 domains, 0 DSSs</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DSS total 1,475 = DSS_View Measurement_Specs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62"/>
+          <t xml:space="preserve">  excluded: 2 domains, 364 DSSs</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  no consumer class assigned: 21 domains, 238 DSSs</t>
+        </is>
+      </c>
+    </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>CHECKS (the run fails otherwise)</t>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  not a Findings domain: 26 domains, 211 DSSs</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Every domain in a Findings file is in that consumer's computed scope.</t>
+          <t xml:space="preserve">  no content: 1 domains, 0 DSSs</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Every covered domain has all its DSS_View DSSs in its Findings file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>Every domain with content is in SDTM_Domain_Metadata; no domain is in two consumer classes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67"/>
+          <t xml:space="preserve">  DSS total 1,475 = DSS_View Measurement_Specs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>CHECKS (the run fails otherwise)</t>
+        </is>
+      </c>
+    </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>HEADER COLOUR CONVENTION</t>
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Every domain in a Findings file is in that consumer's computed scope.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
+          <t>Every covered domain has all its DSS_View DSSs in its Findings file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Every domain with content is in SDTM_Domain_Metadata; no domain is in two consumer classes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71"/>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>HEADER COLOUR CONVENTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
           <t>Green = SDTM-CT side (TESTCD_Count). Yellow = COSMoS side (DSS_Count). Grey = keys, metadata, status.</t>
         </is>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
+    <row r="74"/>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>Not an official CDISC product.</t>
         </is>
@@ -914,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -927,8 +955,9 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -984,10 +1013,15 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
+          <t>DSS_Codelists</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Domain_Notes</t>
         </is>
@@ -1039,7 +1073,8 @@
         </is>
       </c>
       <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="n"/>
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>QRS instrument domain</t>
         </is>
@@ -1091,7 +1126,8 @@
         </is>
       </c>
       <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="7" t="n"/>
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>QRS instrument domain</t>
         </is>
@@ -1143,7 +1179,8 @@
         </is>
       </c>
       <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="7" t="n"/>
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>QRS instrument domain</t>
         </is>
@@ -1196,6 +1233,7 @@
       </c>
       <c r="K5" s="7" t="n"/>
       <c r="L5" s="7" t="n"/>
+      <c r="M5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -1244,6 +1282,7 @@
       </c>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1291,7 +1330,8 @@
         </is>
       </c>
       <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Body System Findings domain (introduced SDTMIG v3.3, 2018). COSMoS BC/DSS coverage added in 2026-03 package: 135 DSS, primarily pulmonary function and respiratory mechanics.</t>
         </is>
@@ -1344,6 +1384,7 @@
       </c>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1392,6 +1433,7 @@
       </c>
       <c r="K9" s="7" t="n"/>
       <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -1440,6 +1482,7 @@
       </c>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1488,6 +1531,7 @@
       </c>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1534,12 +1578,13 @@
           <t>Measurement_Findings (Test_Identity)</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>COSMoS has no DSS for the domain: test identity only</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>TAUG-CV</t>
         </is>
@@ -1590,12 +1635,13 @@
           <t>Specimen_Findings (Test_Identity)</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>COSMoS has no DSS for the domain: test identity only</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="M13" s="7" t="inlineStr">
         <is>
           <t>From SDTMIG-PGx v1.0</t>
         </is>
@@ -1646,12 +1692,13 @@
           <t>Specimen_Findings (Test_Identity)</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>COSMoS has no DSS for the domain: test identity only</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>New in v3.4</t>
         </is>
@@ -1702,12 +1749,13 @@
           <t>Specimen_Findings (Test_Identity)</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="inlineStr">
         <is>
           <t>COSMoS has no DSS for the domain: test identity only</t>
         </is>
       </c>
-      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1754,12 +1802,13 @@
           <t>none in these files</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="inlineStr">
         <is>
           <t>No test codes in SDTM_Test_Identity and no COSMoS DSS (see Domain_Notes)</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>SDTMIG v3.4 binds no codelist to PCTESTCD (the analyte is sponsor-defined), so SDTM_Test_Identity has no PC rows.</t>
         </is>
@@ -1810,12 +1859,13 @@
           <t>none in these files</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>No test codes in SDTM_Test_Identity and no COSMoS DSS (see Domain_Notes)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr">
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Paired with PC. PPTESTCD is bound to PKPARMCD (C85839), which SDTM_CT_Extract does not read by decision (its section 5b), so SDTM_Test_Identity has no PP rows.</t>
         </is>
@@ -1864,10 +1914,15 @@
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
+          <t>GENSMP, GFANMET, GFTEST, GFTESTCD, GFTSDTL, INHERTGF, METHOD, SYMTYPGF, UNIT</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
           <t>Excluded from Specimen_Findings (GF-1, GF-2): Test-detail-driven, not specimen-driven: the DSSs of one BC differ by test detail (TSTDTL). The March 2026 analysis recorded it as scale-driven.</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
         <is>
           <t>New in v3.4</t>
         </is>
@@ -1916,10 +1971,15 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
+          <t>ISBDAGT, ISFTSDTL, ISTEST, ISTESTCD, METHOD, MICROORG, SPECTYPE</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
           <t>Excluded from Specimen_Findings (IS-1, IS-2): Target-driven, not specimen-driven: the DSSs of one BC differ by binding agent (BDAGNT), the target. The March 2026 analysis found the target only in the DS code.</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>Scope expanded in v3.4</t>
         </is>
@@ -1969,6 +2029,11 @@
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2015,7 +2080,12 @@
         </is>
       </c>
       <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2058,8 +2128,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>DTHDX, DTHDXCD</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2105,6 +2184,11 @@
       <c r="K23" s="7" t="n"/>
       <c r="L23" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Device characteristics, not an observation of the subject: no consumer class.</t>
         </is>
       </c>
@@ -2153,6 +2237,11 @@
       <c r="K24" s="7" t="n"/>
       <c r="L24" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Device settings in use, not an observation of the subject: no consumer class.</t>
         </is>
       </c>
@@ -2201,6 +2290,11 @@
       <c r="K25" s="7" t="n"/>
       <c r="L25" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2246,8 +2340,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="n"/>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>CVFATS, CVFATSCD</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2293,6 +2396,11 @@
       <c r="K27" s="7" t="n"/>
       <c r="L27" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2341,6 +2449,11 @@
       <c r="K28" s="7" t="n"/>
       <c r="L28" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2386,8 +2499,17 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="n"/>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>IECAT</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2433,6 +2555,11 @@
       <c r="K30" s="7" t="n"/>
       <c r="L30" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2481,6 +2608,11 @@
       <c r="K31" s="7" t="n"/>
       <c r="L31" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
           <t>In SDTMIG v3.4 (6.3.7.4). Listed here first on 2026-10-01 from SDTM CT C66734 as a domain not in the IG; corrected 2026-10-12. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2529,6 +2661,11 @@
       <c r="K32" s="7" t="n"/>
       <c r="L32" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
           <t>In SDTMIG v3.4 (6.3.7.5). Listed here first on 2026-10-01 from SDTM CT C66734 as a domain not in the IG; corrected 2026-10-12. Consumer class pending published COSMoS content.</t>
         </is>
       </c>
@@ -2577,6 +2714,11 @@
       <c r="K33" s="7" t="n"/>
       <c r="L33" s="7" t="inlineStr">
         <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
           <t>Not in SDTMIG v3.4. Added 2026-10-01 from SDTM CT C66734 (2026-09-25), which defines it as a findings domain. Tobacco product sample testing, not an observation of the subject: no consumer class.</t>
         </is>
       </c>
@@ -2622,8 +2764,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>RPTEST, RPTESTCD, UNIT</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2666,8 +2817,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>SCTEST, SCTESTCD</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2710,8 +2870,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>SRTEST, SRTESTCD</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2755,7 +2924,12 @@
         </is>
       </c>
       <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2798,8 +2972,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K38" s="7" t="n"/>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>TRTEST, TRTESTCD, UNIT</t>
+        </is>
+      </c>
       <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
@@ -2846,8 +3029,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K39" s="7" t="n"/>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>EVAL, TUIDRS, TUTEST, TUTESTCD</t>
+        </is>
+      </c>
       <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
@@ -2894,8 +3086,17 @@
           <t>SDTM_Test_Identity (Test Codes); DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="7" t="n"/>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>SPECTYPE, URNSTS, URNSTSCD</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>No consumer rule places it: Specimen_Based = No, Measurement = No, not in Instrument_Domain_Rules</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2940,6 +3141,7 @@
       </c>
       <c r="K41" s="7" t="n"/>
       <c r="L41" s="7" t="n"/>
+      <c r="M41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2984,6 +3186,7 @@
       </c>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="7" t="n"/>
+      <c r="M42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3026,8 +3229,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="inlineStr">
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>BEDECOD</t>
+        </is>
+      </c>
+      <c r="L43" s="7" t="n"/>
+      <c r="M43" s="7" t="inlineStr">
         <is>
           <t>From SDTMIG-PGx v1.0. Events: specimen handling (collection, culturing, preparation, transport, storage in its COSMoS DSSs). Parent and derived specimens are related in RELSPEC (sheet Non_Observation_Datasets).</t>
         </is>
@@ -3076,6 +3284,7 @@
       </c>
       <c r="K44" s="7" t="n"/>
       <c r="L44" s="7" t="n"/>
+      <c r="M44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3118,8 +3327,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K45" s="7" t="n"/>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>STENRF</t>
+        </is>
+      </c>
       <c r="L45" s="7" t="n"/>
+      <c r="M45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3164,6 +3378,7 @@
       </c>
       <c r="K46" s="7" t="n"/>
       <c r="L46" s="7" t="n"/>
+      <c r="M46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3208,6 +3423,7 @@
       </c>
       <c r="K47" s="7" t="n"/>
       <c r="L47" s="7" t="n"/>
+      <c r="M47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3250,8 +3466,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K48" s="7" t="n"/>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>DSCAT, DSSCAT, NCOMPLT, OTHEVENT, PROTMLST</t>
+        </is>
+      </c>
       <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3296,6 +3517,7 @@
       </c>
       <c r="K49" s="7" t="n"/>
       <c r="L49" s="7" t="n"/>
+      <c r="M49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3338,8 +3560,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K50" s="7" t="n"/>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>FREQ, FRM, ROUTE, UNIT</t>
+        </is>
+      </c>
       <c r="L50" s="7" t="n"/>
+      <c r="M50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3384,6 +3611,7 @@
       </c>
       <c r="K51" s="7" t="n"/>
       <c r="L51" s="7" t="n"/>
+      <c r="M51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3428,6 +3656,7 @@
       </c>
       <c r="K52" s="7" t="n"/>
       <c r="L52" s="7" t="n"/>
+      <c r="M52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3470,8 +3699,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K53" s="7" t="n"/>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>MHEDTTYP</t>
+        </is>
+      </c>
       <c r="L53" s="7" t="n"/>
+      <c r="M53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3515,7 +3749,8 @@
         </is>
       </c>
       <c r="K54" s="7" t="n"/>
-      <c r="L54" s="7" t="inlineStr">
+      <c r="L54" s="7" t="n"/>
+      <c r="M54" s="7" t="inlineStr">
         <is>
           <t>New in v3.4 scope</t>
         </is>
@@ -3562,8 +3797,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K55" s="7" t="n"/>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>LOC, PROCEDUR</t>
+        </is>
+      </c>
       <c r="L55" s="7" t="n"/>
+      <c r="M55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3608,6 +3848,7 @@
       </c>
       <c r="K56" s="7" t="n"/>
       <c r="L56" s="7" t="n"/>
+      <c r="M56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3652,6 +3893,7 @@
       </c>
       <c r="K57" s="7" t="n"/>
       <c r="L57" s="7" t="n"/>
+      <c r="M57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3696,6 +3938,7 @@
       </c>
       <c r="K58" s="7" t="n"/>
       <c r="L58" s="7" t="n"/>
+      <c r="M58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3740,6 +3983,7 @@
       </c>
       <c r="K59" s="7" t="n"/>
       <c r="L59" s="7" t="n"/>
+      <c r="M59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3784,6 +4028,7 @@
       </c>
       <c r="K60" s="7" t="n"/>
       <c r="L60" s="7" t="n"/>
+      <c r="M60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3828,6 +4073,7 @@
       </c>
       <c r="K61" s="7" t="n"/>
       <c r="L61" s="7" t="n"/>
+      <c r="M61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3872,6 +4118,7 @@
       </c>
       <c r="K62" s="7" t="n"/>
       <c r="L62" s="7" t="n"/>
+      <c r="M62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3916,6 +4163,7 @@
       </c>
       <c r="K63" s="7" t="n"/>
       <c r="L63" s="7" t="n"/>
+      <c r="M63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3959,7 +4207,8 @@
         </is>
       </c>
       <c r="K64" s="7" t="n"/>
-      <c r="L64" s="7" t="inlineStr">
+      <c r="L64" s="7" t="n"/>
+      <c r="M64" s="7" t="inlineStr">
         <is>
           <t>Added 2026-10-12 from SDTMIG v3.4.</t>
         </is>
@@ -4006,8 +4255,13 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K65" s="7" t="n"/>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>TSPARM, TSPARMCD</t>
+        </is>
+      </c>
       <c r="L65" s="7" t="n"/>
+      <c r="M65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4052,6 +4306,7 @@
       </c>
       <c r="K66" s="7" t="n"/>
       <c r="L66" s="7" t="n"/>
+      <c r="M66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4095,14 +4350,15 @@
         </is>
       </c>
       <c r="K67" s="7" t="n"/>
-      <c r="L67" s="7" t="inlineStr">
+      <c r="L67" s="7" t="n"/>
+      <c r="M67" s="7" t="inlineStr">
         <is>
           <t>Added 2026-10-12 from SDTMIG v3.4.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Round 4: flag rules stated, instrument flag sources, none named, gaps 6
Findings ReadMes: the rules behind NCIt_Code_Conflict and
NCIt_Reference_Disagree, including that the reference check is lenient
where a TESTCD has more than one reference code (list computed).
Instrument_Findings: which items are compared against which reference,
with counts. Domain_Coverage: "none named" where DSSs name no codelist.
SDTM_Domain_Metadata: CV note spelled out (by hand). SDTM_Test_Identity
known gap 6 (TESTCD equal to NCIt code, as published). SDTM_Instrument_
Test_Identity gap 3: instrument response codelists are not in the file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzSyuaqVq1B4PFnRpWB
</commit_message>
<xml_diff>
--- a/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
+++ b/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
@@ -555,7 +555,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-29 21:53</t>
+          <t>Generated: 2026-10-29 22:07</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  of their Findings file.</t>
+          <t xml:space="preserve">  of their Findings file. "none named": the DSSs name no codelist in any *_codelist column.</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>TAUG-CV</t>
+          <t>TAUG-CV (CDISC Therapeutic Area User Guide for Cardiovascular Studies)</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,11 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K41" s="7" t="n"/>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>none named</t>
+        </is>
+      </c>
       <c r="L41" s="7" t="n"/>
       <c r="M41" s="7" t="n"/>
     </row>
@@ -3421,7 +3425,11 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K47" s="7" t="n"/>
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>none named</t>
+        </is>
+      </c>
       <c r="L47" s="7" t="n"/>
       <c r="M47" s="7" t="n"/>
     </row>
@@ -3609,7 +3617,11 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K51" s="7" t="n"/>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>none named</t>
+        </is>
+      </c>
       <c r="L51" s="7" t="n"/>
       <c r="M51" s="7" t="n"/>
     </row>
@@ -3936,7 +3948,11 @@
           <t>DSS_View (Measurement_Specs)</t>
         </is>
       </c>
-      <c r="K58" s="7" t="n"/>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>none named</t>
+        </is>
+      </c>
       <c r="L58" s="7" t="n"/>
       <c r="M58" s="7" t="n"/>
     </row>

</xml_diff>

<commit_message>
Codelists bound through value lists; NA terms read as published
- DSS_View writes <slot>_codelist for value-list slots too (was pins only).
  Findings Codelists sheets now carry codelists bound only through value
  lists (e.g. IS: TSTOPOBJ, UNIT).
- Findings files leave out a _codelist column empty on every row
  (core slots excepted).
- Immunogenicity_Findings: TSTOPO known gap replaced; ReadMe states the
  4 CT terms vs the 3 in SDTMIG v3.4 IS Assumption 8.
- Domain_Coverage: shared-codelist check compares terms, not
  referenced_by; codelists in COSMoS_Graph_CT Unresolved (ETHNIC, RACE)
  are labelled "not in pinned SDTM CT" instead of stopping.
- Read CodelistTerms / Codelists sheets with keep_default_na=False so the
  terms NA (NY) and None (three instrument codelists) are kept.
- Docs: Changes_2026-10, landing page, sdtm-findings-graph README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzTvNXpqUBwQJ51pu1N
</commit_message>
<xml_diff>
--- a/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
+++ b/sdtm-findings-graph/machine_actionable/Domain_Coverage.xlsx
@@ -554,7 +554,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-30 12:06</t>
+          <t>Generated: 2026-10-30 23:37</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>DTHDX, DTHDXCD</t>
+          <t>AGEU, DTHDX, DTHDXCD, NY</t>
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>CVFATS, CVFATSCD</t>
+          <t>CVFARS, CVFATS, CVFATSCD, EVAL, METHOD</t>
         </is>
       </c>
       <c r="L26" s="7" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>IECAT</t>
+          <t>IECAT, NY</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>RPTEST, RPTESTCD, UNIT</t>
+          <t>LAT, MODDLV, RPTEST, RPTESTCD, UNIT</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>SCTEST, SCTESTCD</t>
+          <t>LAT, MARISTAT, NY, SCTEST, SCTESTCD, SKINCLAS, UNIT</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="K36" s="7" t="inlineStr">
         <is>
-          <t>SRTEST, SRTESTCD</t>
+          <t>METHOD, NY, SIZE, SRTEST, SRTESTCD, UNIT</t>
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>TRTEST, TRTESTCD, UNIT</t>
+          <t>EVAL, MEDEVAL, METHOD, ND, TRPROPRS, TRTEST, TRTESTCD, UNIT</t>
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>EVAL, TUIDRS, TUTEST, TUTESTCD</t>
+          <t>EVAL, MEDEVAL, METHOD, NY, TUIDRS, TUTEST, TUTESTCD</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>SPECTYPE, URNSTS, URNSTSCD</t>
+          <t>LAT, LOC, METHOD, NY, SPECTYPE, UNIT, URNSTS, URNSTSCD</t>
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>none named</t>
+          <t>NY, STENRF</t>
         </is>
       </c>
       <c r="L41" s="7" t="n"/>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="K45" s="7" t="inlineStr">
         <is>
-          <t>STENRF</t>
+          <t>NY, STENRF, TRTINTNT, TRTSET</t>
         </is>
       </c>
       <c r="L45" s="7" t="n"/>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
-          <t>none named</t>
+          <t>AGEU, ETHNIC (not in pinned SDTM CT), RACE (not in pinned SDTM CT), SEX</t>
         </is>
       </c>
       <c r="L47" s="7" t="n"/>
@@ -3585,7 +3585,7 @@
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>FREQ, FRM, ROUTE, UNIT</t>
+          <t>DIR, FREQ, FRM, LAT, LOC, NY, ROUTE, UNIT</t>
         </is>
       </c>
       <c r="L50" s="7" t="n"/>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="K51" s="7" t="inlineStr">
         <is>
-          <t>none named</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="L51" s="7" t="n"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="K53" s="7" t="inlineStr">
         <is>
-          <t>MHEDTTYP</t>
+          <t>MHEDTTYP, NY, STENRF</t>
         </is>
       </c>
       <c r="L53" s="7" t="n"/>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>LOC, PROCEDUR</t>
+          <t>LAT, LOC, NY, PROCEDUR, TRTINTNT, TRTSET</t>
         </is>
       </c>
       <c r="L55" s="7" t="n"/>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>none named</t>
+          <t>FREQ, NY, STENRF, UNIT</t>
         </is>
       </c>
       <c r="L58" s="7" t="n"/>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="K65" s="7" t="inlineStr">
         <is>
-          <t>TSPARM, TSPARMCD</t>
+          <t>NY, TSPARM, TSPARMCD</t>
         </is>
       </c>
       <c r="L65" s="7" t="n"/>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-30 12:06</t>
+          <t>2026-10-30 23:37</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>a56aee8a1fb3790ecc4a531f0fa32858e13fe7fae6a903c6e5fc7cc0cf3d8357</t>
+          <t>381d57c4f98b53833c0c7907684af28787d142f697a94c39312090a97aff5bd6</t>
         </is>
       </c>
     </row>

</xml_diff>